<commit_message>
V9.1.9 - Update PO templates: remap values to column D for new A-D layouts
</commit_message>
<xml_diff>
--- a/includes/templates/purchase-order-summary-rmb-template.xlsx
+++ b/includes/templates/purchase-order-summary-rmb-template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\garyl\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\stock-order-plugin\includes\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FAEAF9F-4CC0-450B-85D0-903BA4E54CBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{915CF16C-72D0-4CF1-A9AF-01FBF18DC026}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Purchase Order" sheetId="1" r:id="rId1"/>
@@ -20,14 +20,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="28">
   <si>
     <t>Purchase Order</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
     <t>Buyer</t>
   </si>
   <si>
@@ -67,9 +64,6 @@
     <t>Amount (RMB)</t>
   </si>
   <si>
-    <t>Total (RMB)</t>
-  </si>
-  <si>
     <t>Deposit / Balance</t>
   </si>
   <si>
@@ -77,24 +71,6 @@
   </si>
   <si>
     <t>Payment</t>
-  </si>
-  <si>
-    <t>Value</t>
-  </si>
-  <si>
-    <t>Deposit FX (RMB/USD)</t>
-  </si>
-  <si>
-    <t>Deposit (RMB)</t>
-  </si>
-  <si>
-    <t>Deposit (USD)</t>
-  </si>
-  <si>
-    <t>Balance (USD)</t>
-  </si>
-  <si>
-    <t>0 USD = 0 RMB</t>
   </si>
   <si>
     <t xml:space="preserve">Shipping terms: 
@@ -106,12 +82,40 @@
   </si>
   <si>
     <t xml:space="preserve">Contact: </t>
+  </si>
+  <si>
+    <t>USD</t>
+  </si>
+  <si>
+    <t>RMB</t>
+  </si>
+  <si>
+    <t>Deposit</t>
+  </si>
+  <si>
+    <t>Balance</t>
+  </si>
+  <si>
+    <t>Deposit FX (USD/RMB)</t>
+  </si>
+  <si>
+    <t>TBC</t>
+  </si>
+  <si>
+    <t>0.000 USD = 0.000 RMB</t>
+  </si>
+  <si>
+    <t>Total</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="2">
+    <numFmt numFmtId="165" formatCode="[$$-409]#,##0.00"/>
+    <numFmt numFmtId="166" formatCode="[$¥-804]#,##0.00"/>
+  </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
@@ -149,7 +153,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -271,29 +275,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -301,86 +287,79 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -715,335 +694,360 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E31"/>
-  <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:D40"/>
+  <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="20" customWidth="1"/>
-    <col min="3" max="3" width="18.77734375" customWidth="1"/>
-    <col min="4" max="5" width="14.44140625" customWidth="1"/>
+    <col min="1" max="1" width="33.5703125" customWidth="1"/>
+    <col min="2" max="2" width="14.28515625" customWidth="1"/>
+    <col min="3" max="3" width="33.5703125" customWidth="1"/>
+    <col min="4" max="4" width="14.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="14" t="s">
+    <row r="1" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="15"/>
-    </row>
-    <row r="2" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="5" t="s">
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="25"/>
+    </row>
+    <row r="2" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="26" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="27"/>
+      <c r="C2" s="26" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="7"/>
-      <c r="C2" s="5" t="s">
+      <c r="D2" s="27"/>
+    </row>
+    <row r="3" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="29"/>
+      <c r="B3" s="30"/>
+      <c r="C3" s="29"/>
+      <c r="D3" s="30"/>
+    </row>
+    <row r="4" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="10"/>
+      <c r="B4" s="11"/>
+      <c r="C4" s="10"/>
+      <c r="D4" s="16"/>
+    </row>
+    <row r="5" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="12"/>
+      <c r="B5" s="13"/>
+      <c r="C5" s="17"/>
+      <c r="D5" s="18"/>
+    </row>
+    <row r="6" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="12"/>
+      <c r="B6" s="13"/>
+      <c r="C6" s="17"/>
+      <c r="D6" s="18"/>
+    </row>
+    <row r="7" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="12"/>
+      <c r="B7" s="13"/>
+      <c r="C7" s="17"/>
+      <c r="D7" s="18"/>
+    </row>
+    <row r="8" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="14"/>
+      <c r="B8" s="15"/>
+      <c r="C8" s="19"/>
+      <c r="D8" s="20"/>
+    </row>
+    <row r="9" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="29"/>
+      <c r="B9" s="30"/>
+      <c r="C9" s="29"/>
+      <c r="D9" s="30"/>
+    </row>
+    <row r="10" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="29"/>
+      <c r="B10" s="30"/>
+      <c r="C10" s="29"/>
+      <c r="D10" s="30"/>
+    </row>
+    <row r="11" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="29" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="6"/>
-      <c r="E2" s="7"/>
-    </row>
-    <row r="3" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="16"/>
-      <c r="B3" s="23"/>
-      <c r="C3" s="16"/>
-      <c r="D3" s="24"/>
-      <c r="E3" s="23"/>
-    </row>
-    <row r="4" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="22"/>
-      <c r="B4" s="25"/>
-      <c r="C4" s="22"/>
-      <c r="D4" s="26"/>
-      <c r="E4" s="27"/>
-    </row>
-    <row r="5" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="28"/>
-      <c r="B5" s="29"/>
-      <c r="C5" s="30"/>
-      <c r="D5" s="31"/>
-      <c r="E5" s="32"/>
-    </row>
-    <row r="6" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="28"/>
-      <c r="B6" s="29"/>
-      <c r="C6" s="30"/>
-      <c r="D6" s="31"/>
-      <c r="E6" s="32"/>
-    </row>
-    <row r="7" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="28"/>
-      <c r="B7" s="29"/>
-      <c r="C7" s="30"/>
-      <c r="D7" s="31"/>
-      <c r="E7" s="32"/>
-    </row>
-    <row r="8" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="33"/>
-      <c r="B8" s="34"/>
-      <c r="C8" s="35"/>
-      <c r="D8" s="36"/>
-      <c r="E8" s="37"/>
-    </row>
-    <row r="9" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="16"/>
-      <c r="B9" s="23"/>
-      <c r="C9" s="16"/>
-      <c r="D9" s="24"/>
-      <c r="E9" s="23"/>
-    </row>
-    <row r="10" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="16"/>
-      <c r="B10" s="23"/>
-      <c r="C10" s="16"/>
-      <c r="D10" s="24"/>
-      <c r="E10" s="23"/>
-    </row>
-    <row r="11" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="16" t="s">
+      <c r="B11" s="30"/>
+      <c r="C11" s="29" t="s">
+        <v>19</v>
+      </c>
+      <c r="D11" s="30"/>
+    </row>
+    <row r="12" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="10"/>
+      <c r="B12" s="16"/>
+      <c r="C12" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D12" s="16"/>
+    </row>
+    <row r="13" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="17"/>
+      <c r="B13" s="18"/>
+      <c r="C13" s="17"/>
+      <c r="D13" s="18"/>
+    </row>
+    <row r="14" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="17"/>
+      <c r="B14" s="18"/>
+      <c r="C14" s="17"/>
+      <c r="D14" s="18"/>
+    </row>
+    <row r="15" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="17"/>
+      <c r="B15" s="18"/>
+      <c r="C15" s="17"/>
+      <c r="D15" s="18"/>
+    </row>
+    <row r="16" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="17"/>
+      <c r="B16" s="18"/>
+      <c r="C16" s="17"/>
+      <c r="D16" s="18"/>
+    </row>
+    <row r="17" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="19"/>
+      <c r="B17" s="20"/>
+      <c r="C17" s="19"/>
+      <c r="D17" s="20"/>
+    </row>
+    <row r="18" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="26" t="s">
         <v>4</v>
       </c>
-      <c r="B11" s="23"/>
-      <c r="C11" s="16" t="s">
+      <c r="B18" s="28"/>
+      <c r="C18" s="28"/>
+      <c r="D18" s="27"/>
+    </row>
+    <row r="19" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B19" s="9"/>
+      <c r="C19" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D19" s="9"/>
+    </row>
+    <row r="20" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B20" s="9"/>
+      <c r="C20" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D20" s="9"/>
+    </row>
+    <row r="21" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B21" s="9"/>
+      <c r="C21" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D21" s="9"/>
+    </row>
+    <row r="22" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="26" t="s">
+        <v>11</v>
+      </c>
+      <c r="B22" s="28"/>
+      <c r="C22" s="28"/>
+      <c r="D22" s="27"/>
+    </row>
+    <row r="23" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="33" t="s">
+        <v>12</v>
+      </c>
+      <c r="B23" s="34"/>
+      <c r="C23" s="34"/>
+      <c r="D23" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="29"/>
+      <c r="B24" s="31"/>
+      <c r="C24" s="31"/>
+      <c r="D24" s="9"/>
+    </row>
+    <row r="25" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="29"/>
+      <c r="B25" s="31"/>
+      <c r="C25" s="31"/>
+      <c r="D25" s="9"/>
+    </row>
+    <row r="26" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="29"/>
+      <c r="B26" s="31"/>
+      <c r="C26" s="31"/>
+      <c r="D26" s="9"/>
+    </row>
+    <row r="27" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="29"/>
+      <c r="B27" s="31"/>
+      <c r="C27" s="31"/>
+      <c r="D27" s="9"/>
+    </row>
+    <row r="28" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="29"/>
+      <c r="B28" s="31"/>
+      <c r="C28" s="31"/>
+      <c r="D28" s="9"/>
+    </row>
+    <row r="29" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A29" s="29"/>
+      <c r="B29" s="31"/>
+      <c r="C29" s="31"/>
+      <c r="D29" s="9"/>
+    </row>
+    <row r="30" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="29"/>
+      <c r="B30" s="31"/>
+      <c r="C30" s="31"/>
+      <c r="D30" s="9"/>
+    </row>
+    <row r="31" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A31" s="29"/>
+      <c r="B31" s="31"/>
+      <c r="C31" s="31"/>
+      <c r="D31" s="9"/>
+    </row>
+    <row r="32" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A32" s="29"/>
+      <c r="B32" s="31"/>
+      <c r="C32" s="31"/>
+      <c r="D32" s="9"/>
+    </row>
+    <row r="33" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A33" s="29"/>
+      <c r="B33" s="31"/>
+      <c r="C33" s="31"/>
+      <c r="D33" s="9"/>
+    </row>
+    <row r="34" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A34" s="35" t="s">
         <v>27</v>
       </c>
-      <c r="D11" s="24"/>
-      <c r="E11" s="23"/>
-    </row>
-    <row r="12" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="22"/>
-      <c r="B12" s="27"/>
-      <c r="C12" s="22" t="s">
+      <c r="B34" s="36"/>
+      <c r="C34" s="36"/>
+      <c r="D34" s="38">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A35" s="26" t="s">
+        <v>14</v>
+      </c>
+      <c r="B35" s="28"/>
+      <c r="C35" s="28"/>
+      <c r="D35" s="32"/>
+    </row>
+    <row r="36" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A36" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B36" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="C36" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="D36" s="6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A37" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B37" s="37">
+        <v>0</v>
+      </c>
+      <c r="C37" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="D12" s="26"/>
-      <c r="E12" s="27"/>
-    </row>
-    <row r="13" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="30"/>
-      <c r="B13" s="32"/>
-      <c r="C13" s="30"/>
-      <c r="D13" s="31"/>
-      <c r="E13" s="32"/>
-    </row>
-    <row r="14" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="30"/>
-      <c r="B14" s="32"/>
-      <c r="C14" s="30"/>
-      <c r="D14" s="31"/>
-      <c r="E14" s="32"/>
-    </row>
-    <row r="15" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="30"/>
-      <c r="B15" s="32"/>
-      <c r="C15" s="30"/>
-      <c r="D15" s="31"/>
-      <c r="E15" s="32"/>
-    </row>
-    <row r="16" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="30"/>
-      <c r="B16" s="32"/>
-      <c r="C16" s="30"/>
-      <c r="D16" s="31"/>
-      <c r="E16" s="32"/>
-    </row>
-    <row r="17" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="35"/>
-      <c r="B17" s="37"/>
-      <c r="C17" s="35"/>
-      <c r="D17" s="36"/>
-      <c r="E17" s="37"/>
-    </row>
-    <row r="18" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B18" s="6"/>
-      <c r="C18" s="6"/>
-      <c r="D18" s="6"/>
-      <c r="E18" s="7"/>
-    </row>
-    <row r="19" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B19" s="38"/>
-      <c r="C19" s="14" t="s">
-        <v>7</v>
-      </c>
-      <c r="D19" s="15"/>
-      <c r="E19" s="38"/>
-    </row>
-    <row r="20" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B20" s="38"/>
-      <c r="C20" s="14" t="s">
-        <v>9</v>
-      </c>
-      <c r="D20" s="15"/>
-      <c r="E20" s="38"/>
-    </row>
-    <row r="21" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B21" s="38"/>
-      <c r="C21" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="D21" s="15"/>
-      <c r="E21" s="38"/>
-    </row>
-    <row r="22" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="B22" s="6"/>
-      <c r="C22" s="6"/>
-      <c r="D22" s="6"/>
-      <c r="E22" s="7"/>
-    </row>
-    <row r="23" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="B23" s="9"/>
-      <c r="C23" s="9"/>
-      <c r="D23" s="10"/>
-      <c r="E23" s="3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="16"/>
-      <c r="B24" s="24"/>
-      <c r="C24" s="24"/>
-      <c r="D24" s="23"/>
-      <c r="E24" s="38">
+      <c r="D37" s="39">
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="11" t="s">
+    <row r="38" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A38" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B38" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="C38" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="D38" s="39">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A39" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="B25" s="12"/>
-      <c r="C25" s="12"/>
-      <c r="D25" s="13"/>
-      <c r="E25" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="B26" s="6"/>
-      <c r="C26" s="6"/>
-      <c r="D26" s="6"/>
-      <c r="E26" s="39"/>
-    </row>
-    <row r="27" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B27" s="19" t="s">
-        <v>19</v>
-      </c>
-      <c r="C27" s="19" t="s">
-        <v>20</v>
-      </c>
-      <c r="D27" s="19" t="s">
-        <v>19</v>
-      </c>
-      <c r="E27" s="18" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="B28" s="20">
-        <v>0</v>
-      </c>
-      <c r="C28" s="20" t="s">
-        <v>24</v>
-      </c>
-      <c r="D28" s="20">
-        <v>0</v>
-      </c>
-      <c r="E28" s="38">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="B29" s="20">
-        <v>0</v>
-      </c>
-      <c r="C29" s="20" t="s">
-        <v>1</v>
-      </c>
-      <c r="D29" s="20" t="s">
-        <v>1</v>
-      </c>
-      <c r="E29" s="38">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="5" t="s">
+      <c r="B39" s="28"/>
+      <c r="C39" s="28"/>
+      <c r="D39" s="27"/>
+    </row>
+    <row r="40" spans="1:4" ht="46.9" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A40" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="B30" s="6"/>
-      <c r="C30" s="6"/>
-      <c r="D30" s="6"/>
-      <c r="E30" s="7"/>
-    </row>
-    <row r="31" spans="1:5" ht="46.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="21" t="s">
-        <v>25</v>
-      </c>
-      <c r="B31" s="40"/>
-      <c r="C31" s="40"/>
-      <c r="D31" s="40"/>
-      <c r="E31" s="40"/>
+      <c r="B40" s="22"/>
+      <c r="C40" s="22"/>
+      <c r="D40" s="22"/>
     </row>
   </sheetData>
-  <mergeCells count="26">
+  <mergeCells count="32">
+    <mergeCell ref="A29:C29"/>
+    <mergeCell ref="A25:C25"/>
+    <mergeCell ref="A26:C26"/>
+    <mergeCell ref="C12:D17"/>
+    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="A39:D39"/>
+    <mergeCell ref="A35:D35"/>
+    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="A33:C33"/>
+    <mergeCell ref="A34:C34"/>
+    <mergeCell ref="A32:C32"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="A30:C30"/>
+    <mergeCell ref="A24:C24"/>
+    <mergeCell ref="A27:C27"/>
+    <mergeCell ref="A28:C28"/>
     <mergeCell ref="A4:B8"/>
-    <mergeCell ref="C4:E8"/>
-    <mergeCell ref="A31:E31"/>
-    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="C4:D8"/>
+    <mergeCell ref="A40:D40"/>
+    <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:E2"/>
+    <mergeCell ref="C2:D2"/>
     <mergeCell ref="A3:B3"/>
-    <mergeCell ref="C3:E3"/>
-    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="C3:D3"/>
     <mergeCell ref="A9:B9"/>
-    <mergeCell ref="C9:E9"/>
-    <mergeCell ref="C10:E10"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="C10:D10"/>
     <mergeCell ref="A10:B10"/>
     <mergeCell ref="A11:B11"/>
-    <mergeCell ref="C11:E11"/>
+    <mergeCell ref="C11:D11"/>
     <mergeCell ref="A12:B17"/>
-    <mergeCell ref="C12:E17"/>
-    <mergeCell ref="A18:E18"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="A30:E30"/>
-    <mergeCell ref="A26:E26"/>
-    <mergeCell ref="A22:E22"/>
-    <mergeCell ref="A23:D23"/>
-    <mergeCell ref="A24:D24"/>
-    <mergeCell ref="A25:D25"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+  <pageSetup paperSize="9" fitToHeight="0" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
V9.2.3 - xlsx template update bump
</commit_message>
<xml_diff>
--- a/includes/templates/purchase-order-summary-rmb-template.xlsx
+++ b/includes/templates/purchase-order-summary-rmb-template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\stock-order-plugin\includes\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{915CF16C-72D0-4CF1-A9AF-01FBF18DC026}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6D2DE31-AF22-44D1-A197-0B9ED986DC45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -113,8 +113,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="165" formatCode="[$$-409]#,##0.00"/>
-    <numFmt numFmtId="166" formatCode="[$¥-804]#,##0.00"/>
+    <numFmt numFmtId="164" formatCode="[$$-409]#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="[$¥-804]#,##0.00"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -279,7 +279,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -287,36 +287,17 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -331,21 +312,9 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -355,11 +324,54 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -707,264 +719,264 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="25"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="31"/>
     </row>
     <row r="2" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="26" t="s">
+      <c r="A2" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="27"/>
-      <c r="C2" s="26" t="s">
+      <c r="B2" s="16"/>
+      <c r="C2" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="27"/>
+      <c r="D2" s="16"/>
     </row>
     <row r="3" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="29"/>
-      <c r="B3" s="30"/>
-      <c r="C3" s="29"/>
-      <c r="D3" s="30"/>
+      <c r="A3" s="7"/>
+      <c r="B3" s="32"/>
+      <c r="C3" s="7"/>
+      <c r="D3" s="32"/>
     </row>
     <row r="4" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="10"/>
-      <c r="B4" s="11"/>
-      <c r="C4" s="10"/>
-      <c r="D4" s="16"/>
+      <c r="A4" s="8"/>
+      <c r="B4" s="22"/>
+      <c r="C4" s="8"/>
+      <c r="D4" s="9"/>
     </row>
     <row r="5" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="12"/>
-      <c r="B5" s="13"/>
-      <c r="C5" s="17"/>
-      <c r="D5" s="18"/>
+      <c r="A5" s="23"/>
+      <c r="B5" s="24"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="11"/>
     </row>
     <row r="6" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="12"/>
-      <c r="B6" s="13"/>
-      <c r="C6" s="17"/>
-      <c r="D6" s="18"/>
+      <c r="A6" s="23"/>
+      <c r="B6" s="24"/>
+      <c r="C6" s="10"/>
+      <c r="D6" s="11"/>
     </row>
     <row r="7" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="12"/>
-      <c r="B7" s="13"/>
-      <c r="C7" s="17"/>
-      <c r="D7" s="18"/>
+      <c r="A7" s="23"/>
+      <c r="B7" s="24"/>
+      <c r="C7" s="10"/>
+      <c r="D7" s="11"/>
     </row>
     <row r="8" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="14"/>
-      <c r="B8" s="15"/>
-      <c r="C8" s="19"/>
-      <c r="D8" s="20"/>
+      <c r="A8" s="25"/>
+      <c r="B8" s="26"/>
+      <c r="C8" s="12"/>
+      <c r="D8" s="13"/>
     </row>
     <row r="9" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="29"/>
-      <c r="B9" s="30"/>
-      <c r="C9" s="29"/>
-      <c r="D9" s="30"/>
+      <c r="A9" s="7"/>
+      <c r="B9" s="32"/>
+      <c r="C9" s="7"/>
+      <c r="D9" s="32"/>
     </row>
     <row r="10" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="29"/>
-      <c r="B10" s="30"/>
-      <c r="C10" s="29"/>
-      <c r="D10" s="30"/>
+      <c r="A10" s="7"/>
+      <c r="B10" s="32"/>
+      <c r="C10" s="7"/>
+      <c r="D10" s="32"/>
     </row>
     <row r="11" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="29" t="s">
+      <c r="A11" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="B11" s="30"/>
-      <c r="C11" s="29" t="s">
+      <c r="B11" s="32"/>
+      <c r="C11" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="D11" s="30"/>
+      <c r="D11" s="32"/>
     </row>
     <row r="12" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="10"/>
-      <c r="B12" s="16"/>
-      <c r="C12" s="10" t="s">
+      <c r="A12" s="8"/>
+      <c r="B12" s="9"/>
+      <c r="C12" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="D12" s="16"/>
+      <c r="D12" s="9"/>
     </row>
     <row r="13" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="17"/>
-      <c r="B13" s="18"/>
-      <c r="C13" s="17"/>
-      <c r="D13" s="18"/>
+      <c r="A13" s="10"/>
+      <c r="B13" s="11"/>
+      <c r="C13" s="10"/>
+      <c r="D13" s="11"/>
     </row>
     <row r="14" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="17"/>
-      <c r="B14" s="18"/>
-      <c r="C14" s="17"/>
-      <c r="D14" s="18"/>
+      <c r="A14" s="10"/>
+      <c r="B14" s="11"/>
+      <c r="C14" s="10"/>
+      <c r="D14" s="11"/>
     </row>
     <row r="15" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="17"/>
-      <c r="B15" s="18"/>
-      <c r="C15" s="17"/>
-      <c r="D15" s="18"/>
+      <c r="A15" s="10"/>
+      <c r="B15" s="11"/>
+      <c r="C15" s="10"/>
+      <c r="D15" s="11"/>
     </row>
     <row r="16" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="17"/>
-      <c r="B16" s="18"/>
-      <c r="C16" s="17"/>
-      <c r="D16" s="18"/>
+      <c r="A16" s="10"/>
+      <c r="B16" s="11"/>
+      <c r="C16" s="10"/>
+      <c r="D16" s="11"/>
     </row>
     <row r="17" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="19"/>
-      <c r="B17" s="20"/>
-      <c r="C17" s="19"/>
-      <c r="D17" s="20"/>
+      <c r="A17" s="12"/>
+      <c r="B17" s="13"/>
+      <c r="C17" s="12"/>
+      <c r="D17" s="13"/>
     </row>
     <row r="18" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="26" t="s">
+      <c r="A18" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="B18" s="28"/>
-      <c r="C18" s="28"/>
-      <c r="D18" s="27"/>
+      <c r="B18" s="15"/>
+      <c r="C18" s="15"/>
+      <c r="D18" s="16"/>
     </row>
     <row r="19" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B19" s="9"/>
-      <c r="C19" s="5" t="s">
+      <c r="B19" s="41"/>
+      <c r="C19" s="36" t="s">
         <v>6</v>
       </c>
-      <c r="D19" s="9"/>
+      <c r="D19" s="41"/>
     </row>
     <row r="20" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B20" s="9"/>
-      <c r="C20" s="5" t="s">
+      <c r="B20" s="41"/>
+      <c r="C20" s="36" t="s">
         <v>8</v>
       </c>
-      <c r="D20" s="9"/>
+      <c r="D20" s="41"/>
     </row>
     <row r="21" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B21" s="9"/>
-      <c r="C21" s="5" t="s">
+      <c r="B21" s="41"/>
+      <c r="C21" s="36" t="s">
         <v>10</v>
       </c>
-      <c r="D21" s="9"/>
+      <c r="D21" s="41"/>
     </row>
     <row r="22" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="26" t="s">
+      <c r="A22" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="B22" s="28"/>
-      <c r="C22" s="28"/>
-      <c r="D22" s="27"/>
+      <c r="B22" s="15"/>
+      <c r="C22" s="15"/>
+      <c r="D22" s="16"/>
     </row>
     <row r="23" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="33" t="s">
+      <c r="A23" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="B23" s="34"/>
-      <c r="C23" s="34"/>
+      <c r="B23" s="19"/>
+      <c r="C23" s="19"/>
       <c r="D23" s="3" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="29"/>
-      <c r="B24" s="31"/>
-      <c r="C24" s="31"/>
-      <c r="D24" s="9"/>
+      <c r="A24" s="39"/>
+      <c r="B24" s="40"/>
+      <c r="C24" s="40"/>
+      <c r="D24" s="37"/>
     </row>
     <row r="25" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="29"/>
-      <c r="B25" s="31"/>
-      <c r="C25" s="31"/>
-      <c r="D25" s="9"/>
+      <c r="A25" s="39"/>
+      <c r="B25" s="40"/>
+      <c r="C25" s="40"/>
+      <c r="D25" s="37"/>
     </row>
     <row r="26" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="29"/>
-      <c r="B26" s="31"/>
-      <c r="C26" s="31"/>
-      <c r="D26" s="9"/>
+      <c r="A26" s="39"/>
+      <c r="B26" s="40"/>
+      <c r="C26" s="40"/>
+      <c r="D26" s="37"/>
     </row>
     <row r="27" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="29"/>
-      <c r="B27" s="31"/>
-      <c r="C27" s="31"/>
-      <c r="D27" s="9"/>
+      <c r="A27" s="39"/>
+      <c r="B27" s="40"/>
+      <c r="C27" s="40"/>
+      <c r="D27" s="37"/>
     </row>
     <row r="28" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="29"/>
-      <c r="B28" s="31"/>
-      <c r="C28" s="31"/>
-      <c r="D28" s="9"/>
+      <c r="A28" s="39"/>
+      <c r="B28" s="40"/>
+      <c r="C28" s="40"/>
+      <c r="D28" s="37"/>
     </row>
     <row r="29" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="29"/>
-      <c r="B29" s="31"/>
-      <c r="C29" s="31"/>
-      <c r="D29" s="9"/>
+      <c r="A29" s="39"/>
+      <c r="B29" s="40"/>
+      <c r="C29" s="40"/>
+      <c r="D29" s="37"/>
     </row>
     <row r="30" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="29"/>
-      <c r="B30" s="31"/>
-      <c r="C30" s="31"/>
-      <c r="D30" s="9"/>
+      <c r="A30" s="39"/>
+      <c r="B30" s="40"/>
+      <c r="C30" s="40"/>
+      <c r="D30" s="37"/>
     </row>
     <row r="31" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="29"/>
-      <c r="B31" s="31"/>
-      <c r="C31" s="31"/>
-      <c r="D31" s="9"/>
+      <c r="A31" s="39"/>
+      <c r="B31" s="40"/>
+      <c r="C31" s="40"/>
+      <c r="D31" s="37"/>
     </row>
     <row r="32" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="29"/>
-      <c r="B32" s="31"/>
-      <c r="C32" s="31"/>
-      <c r="D32" s="9"/>
+      <c r="A32" s="39"/>
+      <c r="B32" s="40"/>
+      <c r="C32" s="40"/>
+      <c r="D32" s="37"/>
     </row>
     <row r="33" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="29"/>
-      <c r="B33" s="31"/>
-      <c r="C33" s="31"/>
-      <c r="D33" s="9"/>
+      <c r="A33" s="39"/>
+      <c r="B33" s="40"/>
+      <c r="C33" s="40"/>
+      <c r="D33" s="37"/>
     </row>
     <row r="34" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="35" t="s">
+      <c r="A34" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="B34" s="36"/>
-      <c r="C34" s="36"/>
+      <c r="B34" s="21"/>
+      <c r="C34" s="21"/>
       <c r="D34" s="38">
         <v>0</v>
       </c>
     </row>
     <row r="35" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="26" t="s">
+      <c r="A35" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="B35" s="28"/>
-      <c r="C35" s="28"/>
-      <c r="D35" s="32"/>
+      <c r="B35" s="15"/>
+      <c r="C35" s="15"/>
+      <c r="D35" s="17"/>
     </row>
     <row r="36" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B36" s="7" t="s">
+      <c r="B36" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="C36" s="7" t="s">
+      <c r="C36" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="D36" s="6" t="s">
+      <c r="D36" s="5" t="s">
         <v>21</v>
       </c>
     </row>
@@ -972,13 +984,13 @@
       <c r="A37" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B37" s="37">
+      <c r="B37" s="33">
         <v>0</v>
       </c>
-      <c r="C37" s="8" t="s">
+      <c r="C37" s="34" t="s">
         <v>26</v>
       </c>
-      <c r="D37" s="39">
+      <c r="D37" s="35">
         <v>0</v>
       </c>
     </row>
@@ -986,51 +998,34 @@
       <c r="A38" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B38" s="8" t="s">
+      <c r="B38" s="34" t="s">
         <v>25</v>
       </c>
-      <c r="C38" s="8" t="s">
+      <c r="C38" s="34" t="s">
         <v>25</v>
       </c>
-      <c r="D38" s="39">
+      <c r="D38" s="35">
         <v>0</v>
       </c>
     </row>
     <row r="39" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="26" t="s">
+      <c r="A39" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="B39" s="28"/>
-      <c r="C39" s="28"/>
-      <c r="D39" s="27"/>
+      <c r="B39" s="15"/>
+      <c r="C39" s="15"/>
+      <c r="D39" s="16"/>
     </row>
     <row r="40" spans="1:4" ht="46.9" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="21" t="s">
+      <c r="A40" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="B40" s="22"/>
-      <c r="C40" s="22"/>
-      <c r="D40" s="22"/>
+      <c r="B40" s="28"/>
+      <c r="C40" s="28"/>
+      <c r="D40" s="28"/>
     </row>
   </sheetData>
   <mergeCells count="32">
-    <mergeCell ref="A29:C29"/>
-    <mergeCell ref="A25:C25"/>
-    <mergeCell ref="A26:C26"/>
-    <mergeCell ref="C12:D17"/>
-    <mergeCell ref="A18:D18"/>
-    <mergeCell ref="A39:D39"/>
-    <mergeCell ref="A35:D35"/>
-    <mergeCell ref="A22:D22"/>
-    <mergeCell ref="A23:C23"/>
-    <mergeCell ref="A33:C33"/>
-    <mergeCell ref="A34:C34"/>
-    <mergeCell ref="A32:C32"/>
-    <mergeCell ref="A31:C31"/>
-    <mergeCell ref="A30:C30"/>
-    <mergeCell ref="A24:C24"/>
-    <mergeCell ref="A27:C27"/>
-    <mergeCell ref="A28:C28"/>
     <mergeCell ref="A4:B8"/>
     <mergeCell ref="C4:D8"/>
     <mergeCell ref="A40:D40"/>
@@ -1046,6 +1041,23 @@
     <mergeCell ref="A11:B11"/>
     <mergeCell ref="C11:D11"/>
     <mergeCell ref="A12:B17"/>
+    <mergeCell ref="A39:D39"/>
+    <mergeCell ref="A35:D35"/>
+    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="A33:C33"/>
+    <mergeCell ref="A34:C34"/>
+    <mergeCell ref="A32:C32"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="A30:C30"/>
+    <mergeCell ref="A24:C24"/>
+    <mergeCell ref="A27:C27"/>
+    <mergeCell ref="A28:C28"/>
+    <mergeCell ref="A29:C29"/>
+    <mergeCell ref="A25:C25"/>
+    <mergeCell ref="A26:C26"/>
+    <mergeCell ref="C12:D17"/>
+    <mergeCell ref="A18:D18"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" fitToHeight="0" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>

</xml_diff>